<commit_message>
flujo llega a fatca
</commit_message>
<xml_diff>
--- a/cypress/fixtures/CapJuntaDir.xlsx
+++ b/cypress/fixtures/CapJuntaDir.xlsx
@@ -475,8 +475,8 @@
         <v>16</v>
       </c>
       <c r="E2" s="6" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("((LEFT(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""),3))) &amp; ""2 "" &amp; (RIGHT(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""), 10)) "),"0102 1997 33101")</f>
-        <v>0102 1997 33101</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("((LEFT(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""),3))) &amp; ""2 "" &amp; (RIGHT(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""), 10)) "),"0102 1997 33133")</f>
+        <v>0102 1997 33133</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>17</v>

</xml_diff>